<commit_message>
Added Ana and Rohullah
</commit_message>
<xml_diff>
--- a/Worker List.xlsx
+++ b/Worker List.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jxiong\GitCode\TimeData_Processing\TimeData_Processing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDCD28CF-D4E6-466A-9D90-0856487D45E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69D500F2-1D14-4B37-B36E-94F22F9E8E66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4470" yWindow="7170" windowWidth="28800" windowHeight="14835" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7890" yWindow="3075" windowWidth="28800" windowHeight="14835" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="94">
   <si>
     <t>Name</t>
   </si>
@@ -303,13 +303,31 @@
   </si>
   <si>
     <t>N521D5060035</t>
+  </si>
+  <si>
+    <t>Ana Rodriguez</t>
+  </si>
+  <si>
+    <t>Rohullah Naderi</t>
+  </si>
+  <si>
+    <t>EAA2FE84</t>
+  </si>
+  <si>
+    <t>F90B3594</t>
+  </si>
+  <si>
+    <t>N521D5060021</t>
+  </si>
+  <si>
+    <t>N521D5060013</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -335,6 +353,12 @@
     <font>
       <sz val="11"/>
       <color rgb="FF242424"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -423,8 +447,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6D563B1C-36AA-4848-8058-EABF055A9F13}" name="WorkerList" displayName="WorkerList" ref="A1:D29" totalsRowShown="0" headerRowDxfId="0">
-  <autoFilter ref="A1:D29" xr:uid="{6D563B1C-36AA-4848-8058-EABF055A9F13}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6D563B1C-36AA-4848-8058-EABF055A9F13}" name="WorkerList" displayName="WorkerList" ref="A1:D31" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="A1:D31" xr:uid="{6D563B1C-36AA-4848-8058-EABF055A9F13}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{BC46EB32-D445-45FC-8C0C-9E1D8D5CC019}" name="Name"/>
     <tableColumn id="2" xr3:uid="{D157ED81-FA40-4E0E-8131-58D637CEEDB6}" name="Number"/>
@@ -698,7 +722,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D29"/>
+  <dimension ref="A1:D31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.7109375" bestFit="1" customWidth="1"/>
@@ -1118,10 +1142,39 @@
         <v>87</v>
       </c>
     </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>88</v>
+      </c>
+      <c r="B30">
+        <v>1222</v>
+      </c>
+      <c r="C30" t="s">
+        <v>90</v>
+      </c>
+      <c r="D30" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>89</v>
+      </c>
+      <c r="B31">
+        <v>1223</v>
+      </c>
+      <c r="C31" t="s">
+        <v>91</v>
+      </c>
+      <c r="D31" t="s">
+        <v>93</v>
+      </c>
+    </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:C34">
     <sortCondition ref="A1:A34"/>
   </sortState>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <tableParts count="1">
@@ -1131,6 +1184,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000DC8F4689D9E3F4E90AB87244FC81278" ma:contentTypeVersion="3" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="782b18ecfc7f388633e7109c6de2c254">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7f08ef0c-19d2-46df-8915-2428da870300" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2efddd814f80025b03089c394466155d" ns2:_="">
     <xsd:import namespace="7f08ef0c-19d2-46df-8915-2428da870300"/>
@@ -1268,22 +1336,24 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C749C57F-916A-4417-9941-468069112434}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80B02D5E-43A9-4D45-81A7-99DDD9C80623}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{709BA9FE-4172-4036-9FEA-255D70E7A54E}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1299,21 +1369,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80B02D5E-43A9-4D45-81A7-99DDD9C80623}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C749C57F-916A-4417-9941-468069112434}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Added Serial number handling to the front end.
</commit_message>
<xml_diff>
--- a/Worker List.xlsx
+++ b/Worker List.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jxiong\GitCode\TimeData_Processing\TimeData_Processing\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://simcona-my.sharepoint.com/personal/bmiller_simcona_com/Documents/Documents/Code/TimeData_Processing/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61DAD676-64E0-4BC3-88A4-396ABDEAFA5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="13_ncr:1_{61DAD676-64E0-4BC3-88A4-396ABDEAFA5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{22042100-97DA-4C16-82A6-469DEEF64458}"/>
   <bookViews>
-    <workbookView xWindow="4290" yWindow="4290" windowWidth="28800" windowHeight="14835" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-71340" yWindow="-165" windowWidth="23040" windowHeight="13575" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="100">
   <si>
     <t>Name</t>
   </si>
@@ -330,6 +330,15 @@
   </si>
   <si>
     <t>N521D5060006</t>
+  </si>
+  <si>
+    <t>BM-Test</t>
+  </si>
+  <si>
+    <t>543AAE5C</t>
+  </si>
+  <si>
+    <t>N521D060016</t>
   </si>
 </sst>
 </file>
@@ -406,7 +415,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -418,7 +427,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -457,8 +465,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6D563B1C-36AA-4848-8058-EABF055A9F13}" name="WorkerList" displayName="WorkerList" ref="A1:D32" totalsRowShown="0" headerRowDxfId="0">
-  <autoFilter ref="A1:D32" xr:uid="{6D563B1C-36AA-4848-8058-EABF055A9F13}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6D563B1C-36AA-4848-8058-EABF055A9F13}" name="WorkerList" displayName="WorkerList" ref="A1:D33" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="A1:D33" xr:uid="{6D563B1C-36AA-4848-8058-EABF055A9F13}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D32">
     <sortCondition ref="C1:C32"/>
   </sortState>
@@ -735,21 +743,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D32"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:D33"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="20.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.42578125" customWidth="1"/>
-    <col min="3" max="3" width="11.28515625" customWidth="1"/>
-    <col min="4" max="4" width="17.7109375" customWidth="1"/>
-    <col min="5" max="5" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.7265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.453125" customWidth="1"/>
+    <col min="3" max="3" width="11.26953125" customWidth="1"/>
+    <col min="4" max="4" width="17.7265625" customWidth="1"/>
+    <col min="5" max="5" width="19.7265625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="5" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.7265625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -763,7 +771,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>49</v>
       </c>
@@ -777,7 +785,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>37</v>
       </c>
@@ -791,7 +799,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>91</v>
       </c>
@@ -805,7 +813,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>29</v>
       </c>
@@ -819,7 +827,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>57</v>
       </c>
@@ -833,7 +841,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>47</v>
       </c>
@@ -847,7 +855,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>14</v>
       </c>
@@ -861,7 +869,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>26</v>
       </c>
@@ -875,7 +883,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>36</v>
       </c>
@@ -889,7 +897,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>35</v>
       </c>
@@ -903,7 +911,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>77</v>
       </c>
@@ -917,7 +925,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>4</v>
       </c>
@@ -931,7 +939,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>23</v>
       </c>
@@ -945,7 +953,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>79</v>
       </c>
@@ -959,7 +967,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>45</v>
       </c>
@@ -973,7 +981,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>82</v>
       </c>
@@ -987,7 +995,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>76</v>
       </c>
@@ -1001,7 +1009,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>52</v>
       </c>
@@ -1015,7 +1023,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>17</v>
       </c>
@@ -1029,7 +1037,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>32</v>
       </c>
@@ -1043,7 +1051,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>51</v>
       </c>
@@ -1057,7 +1065,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
         <v>40</v>
       </c>
@@ -1071,7 +1079,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24" s="6" t="s">
         <v>20</v>
       </c>
@@ -1085,7 +1093,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>85</v>
       </c>
@@ -1099,8 +1107,8 @@
         <v>89</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="7" t="s">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
         <v>48</v>
       </c>
       <c r="B26">
@@ -1113,7 +1121,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>43</v>
       </c>
@@ -1127,7 +1135,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
         <v>11</v>
       </c>
@@ -1141,7 +1149,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>86</v>
       </c>
@@ -1155,7 +1163,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
         <v>55</v>
       </c>
@@ -1169,7 +1177,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>92</v>
       </c>
@@ -1183,7 +1191,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>78</v>
       </c>
@@ -1195,6 +1203,20 @@
       </c>
       <c r="D32" t="s">
         <v>70</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>97</v>
+      </c>
+      <c r="B33">
+        <v>5678</v>
+      </c>
+      <c r="C33" t="s">
+        <v>98</v>
+      </c>
+      <c r="D33" t="s">
+        <v>99</v>
       </c>
     </row>
   </sheetData>
@@ -1211,6 +1233,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000DC8F4689D9E3F4E90AB87244FC81278" ma:contentTypeVersion="3" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="782b18ecfc7f388633e7109c6de2c254">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7f08ef0c-19d2-46df-8915-2428da870300" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2efddd814f80025b03089c394466155d" ns2:_="">
     <xsd:import namespace="7f08ef0c-19d2-46df-8915-2428da870300"/>
@@ -1348,7 +1376,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -1357,13 +1385,16 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80B02D5E-43A9-4D45-81A7-99DDD9C80623}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{709BA9FE-4172-4036-9FEA-255D70E7A54E}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1381,19 +1412,10 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C749C57F-916A-4417-9941-468069112434}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80B02D5E-43A9-4D45-81A7-99DDD9C80623}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Add Phillip Scheuring to Worker List
</commit_message>
<xml_diff>
--- a/Worker List.xlsx
+++ b/Worker List.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jxiong\GitCode\TimeData_Processing\TimeData_Processing\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bmiller\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{924EC981-829F-4B3E-9652-2067D664C4C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B55D2CF-63DC-472E-8BB7-C147BE8C3213}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="-4380" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$4:$A$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$4:$A$27</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="116">
   <si>
     <t>Name</t>
   </si>
@@ -299,86 +299,101 @@
     <t>N521D5060008</t>
   </si>
   <si>
+    <t>N521D5060011</t>
+  </si>
+  <si>
+    <t>3D5FDEB6</t>
+  </si>
+  <si>
+    <t>N521D5060028</t>
+  </si>
+  <si>
+    <t>AB2DD002</t>
+  </si>
+  <si>
+    <t>N521D5060030</t>
+  </si>
+  <si>
+    <t>8166BF3C</t>
+  </si>
+  <si>
+    <t>N521D5060019</t>
+  </si>
+  <si>
+    <t>AF8446CB</t>
+  </si>
+  <si>
+    <t>N515D5060001</t>
+  </si>
+  <si>
+    <t>CB46D992</t>
+  </si>
+  <si>
+    <t>N445D50044</t>
+  </si>
+  <si>
+    <t>FE65C71B</t>
+  </si>
+  <si>
+    <t>N521D5060005</t>
+  </si>
+  <si>
+    <t>3ADE41C3</t>
+  </si>
+  <si>
+    <t>N521D5060002</t>
+  </si>
+  <si>
+    <t>EC44ACBC</t>
+  </si>
+  <si>
+    <t>N521D5060026</t>
+  </si>
+  <si>
+    <t>N521D5060018</t>
+  </si>
+  <si>
+    <t>04A5CF2B</t>
+  </si>
+  <si>
+    <t>N521D5060001</t>
+  </si>
+  <si>
+    <t>1AF41C46</t>
+  </si>
+  <si>
+    <t>N521D5060014</t>
+  </si>
+  <si>
+    <t>Lorenzo Marshall</t>
+  </si>
+  <si>
+    <t>Jenna Trifaro</t>
+  </si>
+  <si>
+    <t>Tamzid Mafiq</t>
+  </si>
+  <si>
+    <t>Cole Witko</t>
+  </si>
+  <si>
+    <t>Laura Rodriguez</t>
+  </si>
+  <si>
     <t>0E9D9A52</t>
   </si>
   <si>
-    <t>N521D5060011</t>
-  </si>
-  <si>
-    <t>3D5FDEB6</t>
-  </si>
-  <si>
-    <t>N521D5060028</t>
-  </si>
-  <si>
-    <t>AB2DD002</t>
-  </si>
-  <si>
-    <t>N521D5060030</t>
-  </si>
-  <si>
-    <t>8166BF3C</t>
-  </si>
-  <si>
-    <t>N521D5060019</t>
-  </si>
-  <si>
-    <t>AF8446CB</t>
-  </si>
-  <si>
-    <t>N515D5060001</t>
-  </si>
-  <si>
-    <t>CB46D992</t>
-  </si>
-  <si>
-    <t>N445D50044</t>
-  </si>
-  <si>
-    <t>FE65C71B</t>
-  </si>
-  <si>
-    <t>N521D5060005</t>
-  </si>
-  <si>
-    <t>3ADE41C3</t>
-  </si>
-  <si>
-    <t>N521D5060002</t>
-  </si>
-  <si>
-    <t>EC44ACBC</t>
-  </si>
-  <si>
-    <t>N521D5060026</t>
-  </si>
-  <si>
-    <t>N521D5060018</t>
-  </si>
-  <si>
-    <t>04A5CF2B</t>
-  </si>
-  <si>
-    <t>N521D5060001</t>
-  </si>
-  <si>
-    <t>1AF41C46</t>
-  </si>
-  <si>
-    <t>N521D5060014</t>
-  </si>
-  <si>
-    <t>Lorenzo Marshall</t>
-  </si>
-  <si>
-    <t>Gary Horton</t>
+    <t>Joseph Torres</t>
+  </si>
+  <si>
+    <t>Phillip Scheuring</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -410,6 +425,13 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -448,7 +470,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -461,6 +483,10 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -503,8 +529,8 @@
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6D563B1C-36AA-4848-8058-EABF055A9F13}" name="WorkerList" displayName="WorkerList" ref="A1:D41" totalsRowShown="0" headerRowDxfId="0">
   <autoFilter ref="A1:D41" xr:uid="{6D563B1C-36AA-4848-8058-EABF055A9F13}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D27">
-    <sortCondition ref="A1:A27"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D26">
+    <sortCondition ref="A1:A26"/>
   </sortState>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{BC46EB32-D445-45FC-8C0C-9E1D8D5CC019}" name="Name"/>
@@ -780,20 +806,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D41"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="20.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.42578125" customWidth="1"/>
-    <col min="3" max="3" width="11.28515625" customWidth="1"/>
-    <col min="4" max="4" width="17.7109375" customWidth="1"/>
-    <col min="5" max="5" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.7265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.453125" customWidth="1"/>
+    <col min="3" max="3" width="11.26953125" customWidth="1"/>
+    <col min="4" max="4" width="17.7265625" customWidth="1"/>
+    <col min="5" max="5" width="19.7265625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="5" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.7265625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -807,21 +833,15 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" s="4">
-        <v>1097</v>
-      </c>
-      <c r="C2" s="2" t="s">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="C2" s="9" t="s">
         <v>5</v>
       </c>
       <c r="D2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>7</v>
       </c>
@@ -835,7 +855,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -849,7 +869,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>13</v>
       </c>
@@ -863,7 +883,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>75</v>
       </c>
@@ -877,7 +897,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -891,7 +911,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>19</v>
       </c>
@@ -905,399 +925,435 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>69</v>
-      </c>
-      <c r="B9">
-        <v>1220</v>
-      </c>
-      <c r="C9" t="s">
-        <v>70</v>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" s="4">
+        <v>1190</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>23</v>
       </c>
       <c r="D9" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B10" s="4">
-        <v>1190</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="C10" s="8" t="s">
+        <v>26</v>
       </c>
       <c r="D10" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
+        <v>65</v>
+      </c>
+      <c r="B11">
+        <v>1180</v>
+      </c>
+      <c r="C11" t="s">
+        <v>58</v>
+      </c>
+      <c r="D11" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12">
+        <v>1169</v>
+      </c>
+      <c r="C12" t="s">
+        <v>64</v>
+      </c>
+      <c r="D12" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="C13" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="D13" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14">
+        <v>1147</v>
+      </c>
+      <c r="C14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D14" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B15" s="4">
+        <v>1088</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="D15" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>36</v>
+      </c>
+      <c r="B16">
+        <v>1171</v>
+      </c>
+      <c r="C16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D16" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A17" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B17" s="4">
+        <v>1182</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D17" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A18" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B18" s="4">
+        <v>1174</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D18" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A19" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="B19">
+        <v>1132</v>
+      </c>
+      <c r="C19" t="s">
+        <v>80</v>
+      </c>
+      <c r="D19" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>42</v>
+      </c>
+      <c r="B20">
+        <v>1165</v>
+      </c>
+      <c r="C20" t="s">
+        <v>43</v>
+      </c>
+      <c r="D20" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>72</v>
+      </c>
+      <c r="B21">
+        <v>1223</v>
+      </c>
+      <c r="C21" t="s">
+        <v>73</v>
+      </c>
+      <c r="D21" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>44</v>
+      </c>
+      <c r="B22">
+        <v>1168</v>
+      </c>
+      <c r="C22" t="s">
+        <v>62</v>
+      </c>
+      <c r="D22" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>45</v>
+      </c>
+      <c r="B23">
+        <v>1116</v>
+      </c>
+      <c r="C23" t="s">
+        <v>46</v>
+      </c>
+      <c r="D23" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A24" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B24" s="4">
+        <v>1134</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D24" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>66</v>
+      </c>
+      <c r="B25">
+        <v>1159</v>
+      </c>
+      <c r="C25" t="s">
+        <v>60</v>
+      </c>
+      <c r="D25" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="C26" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="D26" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>108</v>
+      </c>
+      <c r="B27">
+        <v>1227</v>
+      </c>
+      <c r="C27" t="s">
+        <v>82</v>
+      </c>
+      <c r="D27" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>115</v>
+      </c>
+      <c r="B28">
+        <v>1234</v>
+      </c>
+      <c r="C28" t="s">
+        <v>84</v>
+      </c>
+      <c r="D28" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>112</v>
+      </c>
+      <c r="B29">
+        <v>1232</v>
+      </c>
+      <c r="C29" t="s">
+        <v>113</v>
+      </c>
+      <c r="D29" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>29</v>
+      </c>
+      <c r="B30">
+        <v>1125</v>
+      </c>
+      <c r="C30" t="s">
+        <v>87</v>
+      </c>
+      <c r="D30" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A31" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B31" s="4">
+        <v>1097</v>
+      </c>
+      <c r="C31" t="s">
+        <v>89</v>
+      </c>
+      <c r="D31" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>110</v>
+      </c>
+      <c r="B32">
+        <v>1230</v>
+      </c>
+      <c r="C32" t="s">
+        <v>91</v>
+      </c>
+      <c r="D32" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>111</v>
+      </c>
+      <c r="B33">
+        <v>1231</v>
+      </c>
+      <c r="C33" t="s">
+        <v>93</v>
+      </c>
+      <c r="D33" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>109</v>
+      </c>
+      <c r="B34">
+        <v>1229</v>
+      </c>
+      <c r="C34" t="s">
+        <v>95</v>
+      </c>
+      <c r="D34" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
         <v>25</v>
       </c>
-      <c r="B11">
+      <c r="B35">
         <v>1166</v>
       </c>
-      <c r="C11" t="s">
-        <v>26</v>
-      </c>
-      <c r="D11" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>65</v>
-      </c>
-      <c r="B12">
-        <v>1180</v>
-      </c>
-      <c r="C12" t="s">
-        <v>58</v>
-      </c>
-      <c r="D12" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>28</v>
-      </c>
-      <c r="B13">
-        <v>1169</v>
-      </c>
-      <c r="C13" t="s">
-        <v>64</v>
-      </c>
-      <c r="D13" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>29</v>
-      </c>
-      <c r="B14">
-        <v>1125</v>
-      </c>
-      <c r="C14" t="s">
-        <v>57</v>
-      </c>
-      <c r="D14" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>30</v>
-      </c>
-      <c r="B15">
-        <v>1147</v>
-      </c>
-      <c r="C15" t="s">
-        <v>31</v>
-      </c>
-      <c r="D15" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="B16" s="4">
-        <v>1088</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="D16" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>36</v>
-      </c>
-      <c r="B17">
-        <v>1171</v>
-      </c>
-      <c r="C17" t="s">
-        <v>37</v>
-      </c>
-      <c r="D17" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="B18" s="4">
-        <v>1182</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="D18" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="B19" s="4">
-        <v>1174</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="D19" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="B20">
-        <v>1132</v>
-      </c>
-      <c r="C20" t="s">
-        <v>80</v>
-      </c>
-      <c r="D20" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>42</v>
-      </c>
-      <c r="B21">
-        <v>1165</v>
-      </c>
-      <c r="C21" t="s">
-        <v>43</v>
-      </c>
-      <c r="D21" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>72</v>
-      </c>
-      <c r="B22">
-        <v>1223</v>
-      </c>
-      <c r="C22" t="s">
-        <v>73</v>
-      </c>
-      <c r="D22" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>44</v>
-      </c>
-      <c r="B23">
-        <v>1168</v>
-      </c>
-      <c r="C23" t="s">
-        <v>62</v>
-      </c>
-      <c r="D23" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>45</v>
-      </c>
-      <c r="B24">
-        <v>1116</v>
-      </c>
-      <c r="C24" t="s">
-        <v>46</v>
-      </c>
-      <c r="D24" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="B25" s="4">
-        <v>1134</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="D25" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>66</v>
-      </c>
-      <c r="B26">
-        <v>1159</v>
-      </c>
-      <c r="C26" t="s">
-        <v>60</v>
-      </c>
-      <c r="D26" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>50</v>
-      </c>
-      <c r="B27">
-        <v>1185</v>
-      </c>
-      <c r="C27" t="s">
-        <v>67</v>
-      </c>
-      <c r="D27" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>109</v>
-      </c>
-      <c r="B28">
-        <v>1227</v>
-      </c>
-      <c r="C28" t="s">
-        <v>82</v>
-      </c>
-      <c r="D28" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C29" t="s">
-        <v>84</v>
-      </c>
-      <c r="D29" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C30" t="s">
-        <v>86</v>
-      </c>
-      <c r="D30" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C31" t="s">
-        <v>88</v>
-      </c>
-      <c r="D31" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C32" t="s">
-        <v>90</v>
-      </c>
-      <c r="D32" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C33" t="s">
-        <v>92</v>
-      </c>
-      <c r="D33" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C34" t="s">
-        <v>94</v>
-      </c>
-      <c r="D34" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C35" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D35" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
+        <v>114</v>
+      </c>
+      <c r="B36">
+        <v>1233</v>
+      </c>
       <c r="C36" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D36" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
       <c r="C37" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D37" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C38" t="s">
         <v>102</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="C38" s="7">
+        <v>70626308</v>
       </c>
       <c r="D38" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C39" s="7">
-        <v>70626308</v>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
+        <v>50</v>
+      </c>
+      <c r="B39">
+        <v>1185</v>
+      </c>
+      <c r="C39" t="s">
+        <v>104</v>
       </c>
       <c r="D39" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C40" t="s">
         <v>105</v>
       </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="C40" s="8" t="s">
+        <v>70</v>
+      </c>
       <c r="D40" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A41" t="s">
+        <v>69</v>
+      </c>
+      <c r="B41">
+        <v>1220</v>
+      </c>
+      <c r="C41" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
-        <v>110</v>
-      </c>
-      <c r="B41">
-        <v>1226</v>
-      </c>
-      <c r="C41" t="s">
+      <c r="D41" t="s">
         <v>107</v>
       </c>
-      <c r="D41" t="s">
-        <v>108</v>
-      </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:C28">
-    <sortCondition ref="A1:A28"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:C27">
+    <sortCondition ref="A1:A27"/>
   </sortState>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
New Users per Dan
</commit_message>
<xml_diff>
--- a/Worker List.xlsx
+++ b/Worker List.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://iewc-my.sharepoint.com/personal/bmiller_iewc_com/Documents/Documents/Code/TimeData_Processing/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{57A4C7CF-F123-4D27-A830-3240B1810FC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A91749A9-51DC-4D3E-B737-B5FF59A9ED6A}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="13_ncr:1_{57A4C7CF-F123-4D27-A830-3240B1810FC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8642AE85-B56B-442A-BB59-A1284AB395B5}"/>
   <bookViews>
-    <workbookView xWindow="-80010" yWindow="4245" windowWidth="32400" windowHeight="17250" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-37230" yWindow="2175" windowWidth="32400" windowHeight="17250" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -368,12 +368,6 @@
     <t>Tamzid Mafiq</t>
   </si>
   <si>
-    <t>Cole Witko</t>
-  </si>
-  <si>
-    <t>Laura Rodriguez</t>
-  </si>
-  <si>
     <t>0E9D9A52</t>
   </si>
   <si>
@@ -383,7 +377,13 @@
     <t>Phillip Scheuring</t>
   </si>
   <si>
-    <t xml:space="preserve">Hassam Hussain </t>
+    <t>Craig Hawkins</t>
+  </si>
+  <si>
+    <t>David Riggsbee</t>
+  </si>
+  <si>
+    <t>Tyler Bernard</t>
   </si>
 </sst>
 </file>
@@ -1172,7 +1172,7 @@
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="B28">
         <v>1234</v>
@@ -1186,13 +1186,13 @@
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="B29">
         <v>1232</v>
       </c>
       <c r="C29" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="D29" t="s">
         <v>84</v>
@@ -1242,7 +1242,7 @@
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="B33">
         <v>1231</v>
@@ -1284,7 +1284,7 @@
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="B36">
         <v>1233</v>
@@ -1360,6 +1360,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000DC8F4689D9E3F4E90AB87244FC81278" ma:contentTypeVersion="3" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="782b18ecfc7f388633e7109c6de2c254">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7f08ef0c-19d2-46df-8915-2428da870300" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2efddd814f80025b03089c394466155d" ns2:_="">
     <xsd:import namespace="7f08ef0c-19d2-46df-8915-2428da870300"/>
@@ -1497,22 +1512,24 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80B02D5E-43A9-4D45-81A7-99DDD9C80623}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C749C57F-916A-4417-9941-468069112434}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{709BA9FE-4172-4036-9FEA-255D70E7A54E}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1528,21 +1545,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C749C57F-916A-4417-9941-468069112434}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80B02D5E-43A9-4D45-81A7-99DDD9C80623}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Corrected Worker ID for changes on last two commits.
</commit_message>
<xml_diff>
--- a/Worker List.xlsx
+++ b/Worker List.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://iewc-my.sharepoint.com/personal/bmiller_iewc_com/Documents/Documents/Code/TimeData_Processing/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="13_ncr:1_{57A4C7CF-F123-4D27-A830-3240B1810FC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A56B7BC8-7FA2-4AB2-ADC0-78B12EF5C8A8}"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="13_ncr:1_{57A4C7CF-F123-4D27-A830-3240B1810FC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CACF93F8-AE3B-4E1C-9079-39467606785F}"/>
   <bookViews>
-    <workbookView xWindow="-37230" yWindow="2175" windowWidth="32400" windowHeight="17250" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-32835" yWindow="1965" windowWidth="29355" windowHeight="18030" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1189,7 +1189,7 @@
         <v>112</v>
       </c>
       <c r="B29">
-        <v>1232</v>
+        <v>1238</v>
       </c>
       <c r="C29" t="s">
         <v>108</v>
@@ -1231,7 +1231,7 @@
         <v>114</v>
       </c>
       <c r="B32">
-        <v>1230</v>
+        <v>1236</v>
       </c>
       <c r="C32" t="s">
         <v>89</v>
@@ -1245,7 +1245,7 @@
         <v>111</v>
       </c>
       <c r="B33">
-        <v>1231</v>
+        <v>1237</v>
       </c>
       <c r="C33" t="s">
         <v>91</v>
@@ -1301,7 +1301,7 @@
         <v>113</v>
       </c>
       <c r="B37">
-        <v>1235</v>
+        <v>1239</v>
       </c>
       <c r="C37" t="s">
         <v>99</v>
@@ -1360,6 +1360,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000DC8F4689D9E3F4E90AB87244FC81278" ma:contentTypeVersion="3" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="782b18ecfc7f388633e7109c6de2c254">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7f08ef0c-19d2-46df-8915-2428da870300" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2efddd814f80025b03089c394466155d" ns2:_="">
     <xsd:import namespace="7f08ef0c-19d2-46df-8915-2428da870300"/>
@@ -1497,22 +1512,24 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80B02D5E-43A9-4D45-81A7-99DDD9C80623}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C749C57F-916A-4417-9941-468069112434}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{709BA9FE-4172-4036-9FEA-255D70E7A54E}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1528,21 +1545,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C749C57F-916A-4417-9941-468069112434}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80B02D5E-43A9-4D45-81A7-99DDD9C80623}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Several user changes for New Users
</commit_message>
<xml_diff>
--- a/Worker List.xlsx
+++ b/Worker List.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://iewc-my.sharepoint.com/personal/bmiller_iewc_com/Documents/Documents/Code/TimeData_Processing/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="13_ncr:1_{57A4C7CF-F123-4D27-A830-3240B1810FC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CACF93F8-AE3B-4E1C-9079-39467606785F}"/>
+  <xr:revisionPtr revIDLastSave="22" documentId="13_ncr:1_{57A4C7CF-F123-4D27-A830-3240B1810FC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C938A0CD-E22C-4296-9EBA-EB83E3CB4CC0}"/>
   <bookViews>
-    <workbookView xWindow="-32835" yWindow="1965" windowWidth="29355" windowHeight="18030" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-42060" yWindow="1155" windowWidth="32400" windowHeight="17250" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -89,9 +89,6 @@
     <t>N324D5G0116</t>
   </si>
   <si>
-    <t>Dominic Miller</t>
-  </si>
-  <si>
     <t>DBFC40AA</t>
   </si>
   <si>
@@ -134,9 +131,6 @@
     <t>N445D50019</t>
   </si>
   <si>
-    <t>Michael Maksymciw</t>
-  </si>
-  <si>
     <t>D4C6CF96</t>
   </si>
   <si>
@@ -167,9 +161,6 @@
     <t>0489D091</t>
   </si>
   <si>
-    <t>Saad Shamsaldeen</t>
-  </si>
-  <si>
     <t>Sayed Hossiny</t>
   </si>
   <si>
@@ -362,9 +353,6 @@
     <t>Lorenzo Marshall</t>
   </si>
   <si>
-    <t>Jenna Trifaro</t>
-  </si>
-  <si>
     <t>0E9D9A52</t>
   </si>
   <si>
@@ -384,6 +372,18 @@
   </si>
   <si>
     <t>Landen Evans</t>
+  </si>
+  <si>
+    <t>Malia Silfies</t>
+  </si>
+  <si>
+    <t>Cory Yaniro</t>
+  </si>
+  <si>
+    <t>Deztini Moton</t>
+  </si>
+  <si>
+    <t>Omari Norbrun</t>
   </si>
 </sst>
 </file>
@@ -882,49 +882,49 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B6">
         <v>1225</v>
       </c>
       <c r="C6" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="D6" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
+        <v>113</v>
+      </c>
+      <c r="B7">
+        <v>1242</v>
+      </c>
+      <c r="C7" t="s">
         <v>16</v>
       </c>
-      <c r="B7">
-        <v>1175</v>
-      </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>17</v>
-      </c>
-      <c r="D7" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B8">
         <v>1186</v>
       </c>
       <c r="C8" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" t="s">
         <v>20</v>
-      </c>
-      <c r="D8" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B9" s="4">
         <v>1190</v>
@@ -933,283 +933,283 @@
         <v>70626308</v>
       </c>
       <c r="D9" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="C10" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="D10" t="s">
         <v>24</v>
-      </c>
-      <c r="D10" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B11">
         <v>1180</v>
       </c>
       <c r="C11" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="D11" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B12">
         <v>1169</v>
       </c>
       <c r="C12" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="D12" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="C13" s="8" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="D13" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B14">
         <v>1147</v>
       </c>
       <c r="C14" t="s">
+        <v>28</v>
+      </c>
+      <c r="D14" t="s">
         <v>29</v>
-      </c>
-      <c r="D14" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B15" s="4">
+        <v>1241</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D15" t="s">
         <v>31</v>
-      </c>
-      <c r="B15" s="4">
-        <v>1088</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="D15" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B16">
         <v>1171</v>
       </c>
       <c r="C16" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D16" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B17" s="4">
         <v>1182</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D17" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B18" s="4">
         <v>1174</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="D18" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" s="6" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B19">
         <v>1132</v>
       </c>
       <c r="C19" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D19" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B20">
         <v>1165</v>
       </c>
       <c r="C20" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="D20" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B21">
         <v>1223</v>
       </c>
       <c r="C21" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="D21" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>42</v>
+        <v>114</v>
       </c>
       <c r="B22">
-        <v>1168</v>
+        <v>1243</v>
       </c>
       <c r="C22" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="D22" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B23">
         <v>1116</v>
       </c>
       <c r="C23" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D23" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="B24" s="4">
         <v>1134</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="D24" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B25">
         <v>1159</v>
       </c>
       <c r="C25" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="D25" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="C26" s="8" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="D26" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="B27">
         <v>1227</v>
       </c>
       <c r="C27" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D27" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="B28">
         <v>1234</v>
       </c>
       <c r="C28" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="D28" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="B29">
         <v>1238</v>
       </c>
       <c r="C29" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="D29" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B30">
         <v>1125</v>
       </c>
       <c r="C30" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="D30" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.35">
@@ -1220,130 +1220,130 @@
         <v>1097</v>
       </c>
       <c r="C31" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="D31" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="B32">
         <v>1236</v>
       </c>
       <c r="C32" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="D32" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="B33">
         <v>1237</v>
       </c>
       <c r="C33" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D33" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="B34">
-        <v>1229</v>
+        <v>1240</v>
       </c>
       <c r="C34" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="D34" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B35">
         <v>1166</v>
       </c>
       <c r="C35" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D35" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="B36">
         <v>1233</v>
       </c>
       <c r="C36" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="D36" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="B37">
         <v>1239</v>
       </c>
       <c r="C37" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="D37" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="B38">
         <v>1185</v>
       </c>
       <c r="C38" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="D38" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.35">
       <c r="C39" s="8" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="D39" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B40">
         <v>1220</v>
       </c>
       <c r="C40" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D40" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
     </row>
   </sheetData>
@@ -1360,21 +1360,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000DC8F4689D9E3F4E90AB87244FC81278" ma:contentTypeVersion="3" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="782b18ecfc7f388633e7109c6de2c254">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7f08ef0c-19d2-46df-8915-2428da870300" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2efddd814f80025b03089c394466155d" ns2:_="">
     <xsd:import namespace="7f08ef0c-19d2-46df-8915-2428da870300"/>
@@ -1512,24 +1497,22 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80B02D5E-43A9-4D45-81A7-99DDD9C80623}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C749C57F-916A-4417-9941-468069112434}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{709BA9FE-4172-4036-9FEA-255D70E7A54E}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1545,4 +1528,21 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C749C57F-916A-4417-9941-468069112434}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80B02D5E-43A9-4D45-81A7-99DDD9C80623}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>